<commit_message>
update data and format
</commit_message>
<xml_diff>
--- a/wc.xlsx
+++ b/wc.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="65">
   <si>
     <t>Thái Bình</t>
   </si>
@@ -249,7 +249,7 @@
         <b/>
         <color theme="1"/>
       </rPr>
-      <t>Nhật</t>
+      <t>Nhật Bản</t>
     </r>
   </si>
   <si>
@@ -506,7 +506,197 @@
     </r>
   </si>
   <si>
-    <t>Séc - Nam Phi</t>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">Séc - </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>Nam Phi</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>Thuỵ Sĩ</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve"> - Bosina</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>Canada</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve"> - Qatar</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>Mexico</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve"> - Hàn Quốc</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>Mỹ</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve"> - Úc</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>Ma Rốc</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve"> - Scotland</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>Brazil</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve"> - Halti</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">Thổ Nhĩ Kì - </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>Paraguay</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>Hà Lan</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve"> - Thuỵ Điển</t>
+    </r>
+  </si>
+  <si>
+    <t>Đức - Bờ Biển Ngà</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">Ecuador - </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>Curacao</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>Nhật Bản</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve"> - Tuynidi</t>
+    </r>
+  </si>
+  <si>
+    <t>Tây Ban Nha - Ả Rập Xê út</t>
   </si>
   <si>
     <t>Vua đóng góp</t>
@@ -869,91 +1059,91 @@
     <row r="1">
       <c r="B1" s="1">
         <f t="shared" ref="B1:W1" si="1">sum(B3:B113)</f>
-        <v>260</v>
+        <v>440</v>
       </c>
       <c r="C1" s="1">
         <f t="shared" si="1"/>
-        <v>260</v>
+        <v>340</v>
       </c>
       <c r="D1" s="1">
         <f t="shared" si="1"/>
-        <v>240</v>
+        <v>340</v>
       </c>
       <c r="E1" s="1">
         <f t="shared" si="1"/>
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="F1" s="1">
         <f t="shared" si="1"/>
-        <v>280</v>
+        <v>460</v>
       </c>
       <c r="G1" s="1">
         <f t="shared" si="1"/>
-        <v>260</v>
+        <v>360</v>
       </c>
       <c r="H1" s="1">
         <f t="shared" si="1"/>
-        <v>240</v>
+        <v>360</v>
       </c>
       <c r="I1" s="1">
         <f t="shared" si="1"/>
-        <v>260</v>
+        <v>320</v>
       </c>
       <c r="J1" s="1">
         <f t="shared" si="1"/>
-        <v>180</v>
+        <v>280</v>
       </c>
       <c r="K1" s="1">
         <f t="shared" si="1"/>
-        <v>220</v>
+        <v>280</v>
       </c>
       <c r="L1" s="1">
         <f t="shared" si="1"/>
-        <v>280</v>
+        <v>420</v>
       </c>
       <c r="M1" s="1">
         <f t="shared" si="1"/>
-        <v>220</v>
+        <v>340</v>
       </c>
       <c r="N1" s="1">
         <f t="shared" si="1"/>
-        <v>240</v>
+        <v>320</v>
       </c>
       <c r="O1" s="1">
         <f t="shared" si="1"/>
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="P1" s="1">
         <f t="shared" si="1"/>
-        <v>260</v>
+        <v>360</v>
       </c>
       <c r="Q1" s="1">
         <f t="shared" si="1"/>
-        <v>220</v>
+        <v>280</v>
       </c>
       <c r="R1" s="1">
         <f t="shared" si="1"/>
-        <v>240</v>
+        <v>360</v>
       </c>
       <c r="S1" s="1">
         <f t="shared" si="1"/>
-        <v>220</v>
+        <v>320</v>
       </c>
       <c r="T1" s="1">
         <f t="shared" si="1"/>
-        <v>240</v>
+        <v>380</v>
       </c>
       <c r="U1" s="1">
         <f t="shared" si="1"/>
-        <v>300</v>
+        <v>440</v>
       </c>
       <c r="V1" s="1">
         <f t="shared" si="1"/>
-        <v>300</v>
+        <v>420</v>
       </c>
       <c r="W1" s="1">
         <f t="shared" si="1"/>
-        <v>220</v>
+        <v>320</v>
       </c>
     </row>
     <row r="2">
@@ -2074,90 +2264,465 @@
       <c r="A27" s="5" t="s">
         <v>47</v>
       </c>
+      <c r="C27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="D27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="E27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="F27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="G27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="H27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="I27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="L27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="N27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="O27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="P27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="Q27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="R27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="T27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="U27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="V27" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="W27" s="6">
+        <v>20.0</v>
+      </c>
       <c r="X27" s="7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>340</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8"/>
+      <c r="A28" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="G28" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="H28" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="L28" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="M28" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="T28" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="U28" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="V28" s="6">
+        <v>20.0</v>
+      </c>
       <c r="X28" s="7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>160</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8"/>
+      <c r="A29" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B29" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="F29" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="J29" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="L29" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="M29" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="P29" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="R29" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="S29" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="T29" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="U29" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="V29" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="W29" s="6">
+        <v>20.0</v>
+      </c>
       <c r="X29" s="7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>240</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="8"/>
+      <c r="A30" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="C30" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="D30" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="E30" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="G30" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="H30" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="J30" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="L30" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="M30" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="P30" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="Q30" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="R30" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="S30" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="T30" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="U30" s="6">
+        <v>20.0</v>
+      </c>
       <c r="X30" s="7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>300</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8"/>
+      <c r="A31" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="F31" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="H31" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="K31" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="L31" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="W31" s="6">
+        <v>20.0</v>
+      </c>
       <c r="X31" s="7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="8"/>
+      <c r="A32" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="F32" s="6">
+        <v>20.0</v>
+      </c>
       <c r="X32" s="7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="8"/>
+      <c r="A33" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B33" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="F33" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="H33" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="R33" s="6">
+        <v>20.0</v>
+      </c>
       <c r="X33" s="7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="8"/>
+      <c r="A34" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="F34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="I34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="J34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="K34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="L34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="M34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="N34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="O34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="P34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="R34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="S34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="T34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="U34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="V34" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="W34" s="6">
+        <v>20.0</v>
+      </c>
       <c r="X34" s="7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>320</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="8"/>
+      <c r="A35" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B35" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="C35" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="F35" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="T35" s="6">
+        <v>20.0</v>
+      </c>
       <c r="X35" s="7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="8"/>
+      <c r="A36" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="C36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="D36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="E36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="F36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="G36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="H36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="I36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="J36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="K36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="L36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="M36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="N36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="O36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="P36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="Q36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="R36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="S36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="T36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="U36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="V36" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="W36" s="6">
+        <v>20.0</v>
+      </c>
       <c r="X36" s="7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>440</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="8"/>
+      <c r="A37" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D37" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="F37" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="J37" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="M37" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="N37" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="O37" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="S37" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="U37" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="V37" s="6">
+        <v>20.0</v>
+      </c>
       <c r="X37" s="7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>180</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="8"/>
+      <c r="A38" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B38" s="6">
+        <v>20.0</v>
+      </c>
+      <c r="G38" s="6">
+        <v>20.0</v>
+      </c>
       <c r="X38" s="7">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="8"/>
+      <c r="A39" s="5" t="s">
+        <v>59</v>
+      </c>
       <c r="X39" s="7">
         <f t="shared" si="2"/>
         <v>0</v>
@@ -2658,13 +3223,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="9" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2">
@@ -2674,26 +3239,26 @@
 2,
 FALSE
 )</f>
-        <v>Chính Đạt</v>
+        <v>Tiến Tùng</v>
       </c>
       <c r="B2" s="7">
-        <v>300.0</v>
+        <v>460.0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="s">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="B3" s="7">
-        <v>300.0</v>
+        <v>440.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B4" s="7">
-        <v>280.0</v>
+        <v>440.0</v>
       </c>
     </row>
     <row r="5">
@@ -2701,23 +3266,23 @@
         <v>10</v>
       </c>
       <c r="B5" s="7">
-        <v>280.0</v>
+        <v>420.0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="10" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="B6" s="7">
-        <v>260.0</v>
+        <v>420.0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="B7" s="7">
-        <v>260.0</v>
+        <v>380.0</v>
       </c>
     </row>
     <row r="8">
@@ -2725,15 +3290,15 @@
         <v>5</v>
       </c>
       <c r="B8" s="7">
-        <v>260.0</v>
+        <v>360.0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="7">
-        <v>260.0</v>
+        <v>360.0</v>
       </c>
     </row>
     <row r="10">
@@ -2741,111 +3306,111 @@
         <v>14</v>
       </c>
       <c r="B10" s="7">
-        <v>260.0</v>
+        <v>360.0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="B11" s="7">
-        <v>240.0</v>
+        <v>360.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B12" s="7">
-        <v>240.0</v>
+        <v>340.0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="B13" s="7">
-        <v>240.0</v>
+        <v>340.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" s="7">
-        <v>240.0</v>
+        <v>340.0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B15" s="7">
-        <v>240.0</v>
+        <v>320.0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B16" s="7">
-        <v>240.0</v>
+        <v>320.0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="B17" s="7">
-        <v>220.0</v>
+        <v>320.0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B18" s="7">
-        <v>220.0</v>
+        <v>320.0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="B19" s="7">
-        <v>220.0</v>
+        <v>300.0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B20" s="7">
-        <v>220.0</v>
+        <v>300.0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="B21" s="7">
-        <v>220.0</v>
+        <v>280.0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="B22" s="7">
-        <v>220.0</v>
+        <v>280.0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B23" s="7">
-        <v>180.0</v>
+        <v>280.0</v>
       </c>
     </row>
     <row r="24">
@@ -2853,20 +3418,20 @@
     </row>
     <row r="25">
       <c r="A25" s="12" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="B25" s="13">
         <f>SUM(B2:B23)</f>
-        <v>5400</v>
+        <v>7740</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="B26" s="13">
         <f>ROUND(B25/22,0)</f>
-        <v>245</v>
+        <v>352</v>
       </c>
     </row>
     <row r="27">

</xml_diff>